<commit_message>
Oppdater 2026-resultater og nettside
</commit_message>
<xml_diff>
--- a/SK Vidar Langdistanse 2026.xlsx
+++ b/SK Vidar Langdistanse 2026.xlsx
@@ -575,7 +575,7 @@
         <v>368</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>38</v>
@@ -641,7 +641,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -679,12 +679,12 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Constantin Rust</t>
+          <t>Constantin Rust *</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -907,12 +907,12 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Andreas Sjurseth</t>
+          <t>Andreas Sjurseth *</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -1021,12 +1021,12 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Fredrik Frossdal</t>
+          <t>Fredrik Frossdal *</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1401,12 +1401,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Øyvind Lie</t>
+          <t>Øyvind Lie *</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -1553,12 +1553,12 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Stein Ellingsen</t>
+          <t>Stein Ellingsen *</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Kristoffer Bugge</t>
+          <t>Kristoffer Bugge *</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -1857,12 +1857,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Tormod Fauske Tho</t>
+          <t>Tormod Fauske Tho *</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -2047,12 +2047,12 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Eskil Engdahl</t>
+          <t>Eskil Engdahl *</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -2161,12 +2161,12 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Ingrid Helene Nyhus</t>
+          <t>Ingrid Helene Nyhus *</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -2351,12 +2351,12 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Jon-Henrik Eskeland</t>
+          <t>Jon-Henrik Eskeland *</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -2465,12 +2465,12 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Elliot Jones</t>
+          <t>Elliot Jones *</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -2959,12 +2959,12 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Vegard Grut</t>
+          <t>Vegard Grut *</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -3605,12 +3605,12 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Ingrid Muri</t>
+          <t>Ingrid Muri *</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
@@ -3643,12 +3643,12 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Herborg Hermansen Tveit</t>
+          <t>Herborg Hermansen Tveit *</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
@@ -3681,12 +3681,12 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Håvard Ola Eggen</t>
+          <t>Håvard Ola Eggen *</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
@@ -3757,7 +3757,7 @@
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -4137,12 +4137,12 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Aksel Spence</t>
+          <t>Aksel Spence *</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
@@ -4175,12 +4175,12 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>Erik Flølo</t>
+          <t>Erik Flølo *</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
@@ -4213,12 +4213,12 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>Vilde Dille Øvreeide</t>
+          <t>Vilde Dille Øvreeide *</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -4365,12 +4365,12 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>Ida Christine Østreng</t>
+          <t>Ida Christine Østreng *</t>
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
@@ -4631,12 +4631,12 @@
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>Maren Mohagen</t>
+          <t>Maren Mohagen *</t>
         </is>
       </c>
       <c r="E114" s="6" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>Maria Kongsli Bondestad</t>
+          <t>Maria Kongsli Bondestad *</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr">
@@ -4745,7 +4745,7 @@
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
@@ -4821,7 +4821,7 @@
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
@@ -4935,12 +4935,12 @@
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>Nathalie Moen Balhald</t>
+          <t>Nathalie Moen Balhald *</t>
         </is>
       </c>
       <c r="E122" s="6" t="inlineStr">
@@ -4973,12 +4973,12 @@
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>Tale Glende</t>
+          <t>Tale Glende *</t>
         </is>
       </c>
       <c r="E123" s="6" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
@@ -5125,7 +5125,7 @@
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
@@ -14235,7 +14235,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Sparebank 1 SØR-NORGE Drammen10K</t>
+          <t>Sparebank 1 S?R-NORGE Drammen10K</t>
         </is>
       </c>
     </row>

</xml_diff>